<commit_message>
Update ITU data (2025 edition), auto-generate LaTeX tables/macros, add robustness analyses
- ITU price baskets updated to 2008-2025 Excel (code_prefix filtering)
- Auto-generated descriptive stats table and 109 LaTeX macros from data
- All hardcoded values in manuscript replaced with macro references
- Added period-split, IV robustness, and jackknife analyses
- World Bank control variables updated (GDP, urban pop revisions)
- Fixed broadband price data unchanged; mobile prices reflect basket redefinition
- Removed submission/ folder (consolidated into manuscript/)
</commit_message>
<xml_diff>
--- a/data/interim/data_catalog.xlsx
+++ b/data/interim/data_catalog.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,57 +417,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>data_source</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>variable</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>series_code</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>series_name</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>units</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>observations</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>countries</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>year_min</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>year_max</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>value_min</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>value_max</t>
         </is>
@@ -498,7 +486,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>fixed_broadband</t>
+          <t>i154_FBB</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -543,7 +531,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>fixed_broadband</t>
+          <t>i154_FBB</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -588,7 +576,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>fixed_broadband</t>
+          <t>i154_FBB</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -633,7 +621,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>data_only mobile_broadband</t>
+          <t>i271mb</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -647,13 +635,13 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>394</v>
+        <v>231</v>
       </c>
       <c r="G5" t="n">
         <v>33</v>
       </c>
       <c r="H5" t="n">
-        <v>2013</v>
+        <v>2018</v>
       </c>
       <c r="I5" t="n">
         <v>2024</v>
@@ -662,7 +650,7 @@
         <v>1.74</v>
       </c>
       <c r="K5" t="n">
-        <v>41.33</v>
+        <v>48.45</v>
       </c>
     </row>
     <row r="6">
@@ -678,7 +666,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>data_only mobile_broadband</t>
+          <t>i271mb</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -692,22 +680,22 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>394</v>
+        <v>231</v>
       </c>
       <c r="G6" t="n">
         <v>33</v>
       </c>
       <c r="H6" t="n">
-        <v>2013</v>
+        <v>2018</v>
       </c>
       <c r="I6" t="n">
         <v>2024</v>
       </c>
       <c r="J6" t="n">
-        <v>0.09</v>
+        <v>0.12</v>
       </c>
       <c r="K6" t="n">
-        <v>3.86</v>
+        <v>2.62</v>
       </c>
     </row>
     <row r="7">
@@ -723,7 +711,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>data_only mobile_broadband</t>
+          <t>i271mb</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -737,13 +725,13 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>386</v>
+        <v>229</v>
       </c>
       <c r="G7" t="n">
         <v>33</v>
       </c>
       <c r="H7" t="n">
-        <v>2013</v>
+        <v>2018</v>
       </c>
       <c r="I7" t="n">
         <v>2024</v>
@@ -752,7 +740,7 @@
         <v>4.54</v>
       </c>
       <c r="K7" t="n">
-        <v>35.93</v>
+        <v>56.86</v>
       </c>
     </row>
     <row r="8">
@@ -769,23 +757,23 @@
       <c r="C8" t="inlineStr">
         <is>
           <t xml:space="preserve">    i4213tfbb
-Name: 0, dtype: object</t>
+Name: 0, dtype: str</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
           <t xml:space="preserve">    i4213tfbb
-Name: 0, dtype: object</t>
+Name: 0, dtype: str</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
           <t xml:space="preserve">    per 100 people
-Name: 0, dtype: object</t>
+Name: 0, dtype: str</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="G8" t="n">
         <v>33</v>
@@ -800,7 +788,7 @@
         <v>93586</v>
       </c>
       <c r="K8" t="n">
-        <v>38561700</v>
+        <v>38561677</v>
       </c>
     </row>
     <row r="9">
@@ -817,23 +805,23 @@
       <c r="C9" t="inlineStr">
         <is>
           <t xml:space="preserve">    i992b
-Name: 1, dtype: object</t>
+Name: 1, dtype: str</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
           <t xml:space="preserve">    i992b
-Name: 1, dtype: object</t>
+Name: 1, dtype: str</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
           <t xml:space="preserve">    per 100 people
-Name: 1, dtype: object</t>
+Name: 1, dtype: str</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="G9" t="n">
         <v>33</v>
@@ -865,23 +853,23 @@
       <c r="C10" t="inlineStr">
         <is>
           <t xml:space="preserve">    i99H
-Name: 0, dtype: object</t>
+Name: 0, dtype: str</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
           <t xml:space="preserve">    i99H
-Name: 0, dtype: object</t>
+Name: 0, dtype: str</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
           <t xml:space="preserve">    %
-Name: 0, dtype: object</t>
+Name: 0, dtype: str</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>484</v>
+        <v>495</v>
       </c>
       <c r="G10" t="n">
         <v>33</v>
@@ -913,19 +901,19 @@
       <c r="C11" t="inlineStr">
         <is>
           <t xml:space="preserve">    i4214
-Name: 0, dtype: object</t>
+Name: 0, dtype: str</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
           <t xml:space="preserve">    i4214
-Name: 0, dtype: object</t>
+Name: 0, dtype: str</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
           <t xml:space="preserve">    Mbit/s
-Name: 0, dtype: object</t>
+Name: 0, dtype: str</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -961,19 +949,19 @@
       <c r="C12" t="inlineStr">
         <is>
           <t xml:space="preserve">    i994
-Name: 1, dtype: object</t>
+Name: 1, dtype: str</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
           <t xml:space="preserve">    i994
-Name: 1, dtype: object</t>
+Name: 1, dtype: str</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
           <t xml:space="preserve">    Mbit/s
-Name: 1, dtype: object</t>
+Name: 1, dtype: str</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -992,7 +980,7 @@
         <v>3598.33</v>
       </c>
       <c r="K12" t="n">
-        <v>8047010</v>
+        <v>8047007.94</v>
       </c>
     </row>
     <row r="13">
@@ -1009,19 +997,19 @@
       <c r="C13" t="inlineStr">
         <is>
           <t xml:space="preserve">    i994B
-Name: 2, dtype: object</t>
+Name: 2, dtype: str</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
           <t xml:space="preserve">    i994B
-Name: 2, dtype: object</t>
+Name: 2, dtype: str</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
           <t xml:space="preserve">    Mbit/s
-Name: 2, dtype: object</t>
+Name: 2, dtype: str</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -1037,10 +1025,10 @@
         <v>2014</v>
       </c>
       <c r="J13" t="n">
-        <v>40218.8</v>
+        <v>40218.77</v>
       </c>
       <c r="K13" t="n">
-        <v>18736600</v>
+        <v>18736616.7</v>
       </c>
     </row>
     <row r="14">
@@ -1057,19 +1045,19 @@
       <c r="C14" t="inlineStr">
         <is>
           <t xml:space="preserve">    i994u
-Name: 3, dtype: object</t>
+Name: 3, dtype: str</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
           <t xml:space="preserve">    i994u
-Name: 3, dtype: object</t>
+Name: 3, dtype: str</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Mbit/s
-Name: 3, dtype: object</t>
+Name: 3, dtype: str</t>
         </is>
       </c>
       <c r="F14" t="n">
@@ -1088,7 +1076,7 @@
         <v>9031.379999999999</v>
       </c>
       <c r="K14" t="n">
-        <v>8264960</v>
+        <v>8264958.16</v>
       </c>
     </row>
     <row r="15">
@@ -1105,19 +1093,19 @@
       <c r="C15" t="inlineStr">
         <is>
           <t xml:space="preserve">    i271
-Name: 0, dtype: object</t>
+Name: 0, dtype: str</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
           <t xml:space="preserve">    i271
-Name: 0, dtype: object</t>
+Name: 0, dtype: str</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
           <t xml:space="preserve">    count
-Name: 0, dtype: object</t>
+Name: 0, dtype: str</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -1153,19 +1141,19 @@
       <c r="C16" t="inlineStr">
         <is>
           <t xml:space="preserve">    i911
-Name: 1, dtype: object</t>
+Name: 1, dtype: str</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
           <t xml:space="preserve">    i911
-Name: 1, dtype: object</t>
+Name: 1, dtype: str</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
           <t xml:space="preserve">    count
-Name: 1, dtype: object</t>
+Name: 1, dtype: str</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -1229,7 +1217,7 @@
         <v>2094.47</v>
       </c>
       <c r="K17" t="n">
-        <v>137516.59</v>
+        <v>137781.68</v>
       </c>
     </row>
     <row r="18">
@@ -1409,7 +1397,7 @@
         <v>414508</v>
       </c>
       <c r="K21" t="n">
-        <v>83901923</v>
+        <v>83516593</v>
       </c>
     </row>
     <row r="22">
@@ -1496,10 +1484,10 @@
         <v>2024</v>
       </c>
       <c r="J23" t="n">
-        <v>42.49</v>
+        <v>39.28</v>
       </c>
       <c r="K23" t="n">
-        <v>98.22</v>
+        <v>95.65000000000001</v>
       </c>
     </row>
     <row r="24">
@@ -1664,7 +1652,7 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="G27" t="n">
         <v>33</v>
@@ -1676,7 +1664,7 @@
         <v>2024</v>
       </c>
       <c r="J27" t="n">
-        <v>56.28</v>
+        <v>66.51000000000001</v>
       </c>
       <c r="K27" t="n">
         <v>89.56999999999999</v>
@@ -1889,7 +1877,7 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>464</v>
+        <v>491</v>
       </c>
       <c r="G32" t="n">
         <v>33</v>
@@ -1904,7 +1892,7 @@
         <v>4727643</v>
       </c>
       <c r="K32" t="n">
-        <v>255687490788</v>
+        <v>260043024452</v>
       </c>
     </row>
     <row r="33">
@@ -2024,7 +2012,7 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>460</v>
+        <v>492</v>
       </c>
       <c r="G35" t="n">
         <v>33</v>
@@ -2036,10 +2024,10 @@
         <v>2024</v>
       </c>
       <c r="J35" t="n">
-        <v>31.33</v>
+        <v>31.69</v>
       </c>
       <c r="K35" t="n">
-        <v>96.2</v>
+        <v>93.01000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>